<commit_message>
Time range, metric help, DCF boxes, trend and average lines, screener
- Time range from the sidebar, the graph's range buttons and slider, or drag-to-zoom
- Plain-language hover help for every metric, with how often it updates
- DCF range drawn as a semi-transparent box per quarter; optional typed-in
  dcf_low / dcf_average / dcf_high columns in the manual sheet
- Linear, polynomial and log trend lines, 5/10-year average lines
- Quarterly price as bars with optional value labels
- Screener page with AND conditions on the latest metrics

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LGo2oJ4vcQwb4KKr1wczEc
</commit_message>
<xml_diff>
--- a/templates/manual_entries_template.xlsx
+++ b/templates/manual_entries_template.xlsx
@@ -434,7 +434,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A12"/>
+  <dimension ref="A1:A13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -495,26 +495,33 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>metric: pick from the dropdown; the list with descriptions is on the 'metrics' tab.</t>
+          <t xml:space="preserve">  dcf_low / dcf_average / dcf_high: optional. Type your own range here; it wins over the calculated one.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>ticker: as on the watchlist (AMZN, FTK).</t>
+          <t>metric: pick from the dropdown; the list with descriptions is on the 'metrics' tab.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Manual values always win over automatically extracted ones.</t>
+          <t>ticker: as on the watchlist (AMZN, FTK).</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Manual values always win over automatically extracted ones.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
         <is>
           <t>Don't rename tabs or column headers; the tool reads them by name.</t>
         </is>
@@ -1127,7 +1134,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K1"/>
+  <dimension ref="A1:N1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1141,6 +1148,9 @@
     <col width="16" customWidth="1" min="9" max="9"/>
     <col width="16" customWidth="1" min="10" max="10"/>
     <col width="16" customWidth="1" min="11" max="11"/>
+    <col width="16" customWidth="1" min="12" max="12"/>
+    <col width="16" customWidth="1" min="13" max="13"/>
+    <col width="16" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1195,6 +1205,21 @@
         </is>
       </c>
       <c r="K1" s="3" t="inlineStr">
+        <is>
+          <t>dcf_low</t>
+        </is>
+      </c>
+      <c r="L1" s="3" t="inlineStr">
+        <is>
+          <t>dcf_average</t>
+        </is>
+      </c>
+      <c r="M1" s="3" t="inlineStr">
+        <is>
+          <t>dcf_high</t>
+        </is>
+      </c>
+      <c r="N1" s="3" t="inlineStr">
         <is>
           <t>note</t>
         </is>
@@ -1216,7 +1241,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K7"/>
+  <dimension ref="A1:N8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1356,6 +1381,21 @@
       </c>
       <c r="K6" t="inlineStr">
         <is>
+          <t>dcf_low</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>dcf_average</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>dcf_high</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
           <t>note</t>
         </is>
       </c>
@@ -1398,6 +1438,47 @@
         </is>
       </c>
       <c r="K7" t="inlineStr"/>
+      <c r="L7" t="inlineStr"/>
+      <c r="M7" t="inlineStr"/>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>7 site estimates</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>FTK</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>2026Q4</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr"/>
+      <c r="D8" t="inlineStr"/>
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" t="inlineStr"/>
+      <c r="G8" t="inlineStr"/>
+      <c r="H8" t="inlineStr"/>
+      <c r="I8" t="inlineStr"/>
+      <c r="J8" t="inlineStr"/>
+      <c r="K8" t="n">
+        <v>100</v>
+      </c>
+      <c r="L8" t="n">
+        <v>120</v>
+      </c>
+      <c r="M8" t="n">
+        <v>140</v>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>own range typed in</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>